<commit_message>
minor guideline updates, no version change
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t xml:space="preserve">WORD</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t xml:space="preserve">REF_DIST_ANTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMMENT</t>
   </si>
 </sst>
 </file>
@@ -86,7 +89,7 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -114,7 +117,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE0C2CD"/>
-        <bgColor rgb="FFCCCCFF"/>
+        <bgColor rgb="FFB4C7DC"/>
       </patternFill>
     </fill>
     <fill>
@@ -123,8 +126,14 @@
         <bgColor rgb="FFDEE6EF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB4C7DC"/>
+        <bgColor rgb="FF99CCFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -150,6 +159,13 @@
       <left style="thin"/>
       <right/>
       <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -179,7 +195,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -212,11 +228,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -232,12 +252,16 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -265,7 +289,7 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFE0C2CD"/>
+      <rgbColor rgb="FFB4C7DC"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
@@ -274,7 +298,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFE0C2CD"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -317,11 +341,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="18.89"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="10" min="9" style="0" width="11.54"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="11" min="11" style="0" width="18.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="46.68"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -358,68 +384,73 @@
       <c r="K1" s="7" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="8" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="8"/>
-      <c r="E2" s="9" t="str">
+      <c r="B2" s="9"/>
+      <c r="E2" s="10" t="str">
         <f aca="false">IF(D2="?OLD","!!!","")</f>
         <v/>
       </c>
-      <c r="F2" s="10" t="str">
+      <c r="F2" s="11" t="str">
         <f aca="false">IF(OR(E2="",E2="!!!"),"",IF(NOT(ISNA(VLOOKUP(E2,E$1:E1,1,FALSE()))),"OLD",IF(AND(E2&lt;&gt;"",E2&lt;&gt;"!!!"),"NEW","")))</f>
         <v/>
       </c>
-      <c r="G2" s="11" t="str">
+      <c r="G2" s="12" t="str">
         <f aca="false">IF(OR(E2="",E2="!!!"),"",IF(OR(J2=0,AND(J2=1,K2=1),AND(J2=1,I2="SBJ"),AND(J2=1,I2=0)),"?IN_FOCUS",IF(J2&lt;=2,"?ACTIVATED",IF(J2&lt;&gt;"","?FAMILIAR",IF(F2="NEW",IF(ISNA(VLOOKUP(E2,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
         <v/>
       </c>
-      <c r="H2" s="12" t="str">
+      <c r="H2" s="13" t="str">
         <f aca="false">IF(J2&lt;&gt;1,"",IF(I2="SBJ","CB","?"))</f>
         <v/>
       </c>
-      <c r="I2" s="13" t="str">
+      <c r="I2" s="14" t="str">
         <f aca="false">IF(OR(E2="",E2="!!!",F2="NEW"),"",INDEX(B1:B$2,-1+SUMPRODUCT(MAX(ROW(E1:E$2)*(E2=E1:E$2)))))</f>
         <v/>
       </c>
-      <c r="J2" s="14" t="str">
+      <c r="J2" s="15" t="str">
         <f aca="true">IF(OR(E2="",E2="!!!",F2="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E2)*(E2=E$2:E2)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E1)*(E2=E$1:E1))))))</f>
         <v/>
       </c>
-      <c r="K2" s="14" t="str">
+      <c r="K2" s="15" t="str">
         <f aca="false">IF(OR(E2="",E2="!!!",F2="NEW"),"",INDEX(J$1:J1,SUMPRODUCT(MAX(ROW(E$1:E1)*(E2=E$1:E1)))))</f>
         <v/>
       </c>
+      <c r="L2" s="16"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="8"/>
-      <c r="E3" s="9" t="str">
+      <c r="B3" s="9"/>
+      <c r="E3" s="10" t="str">
         <f aca="false">IF(D3="?OLD","!!!","")</f>
         <v/>
       </c>
-      <c r="F3" s="10" t="str">
+      <c r="F3" s="11" t="str">
         <f aca="false">IF(OR(E3="",E3="!!!"),"",IF(NOT(ISNA(VLOOKUP(E3,E$1:E2,1,FALSE()))),"OLD",IF(AND(E3&lt;&gt;"",E3&lt;&gt;"!!!"),"NEW","")))</f>
         <v/>
       </c>
-      <c r="G3" s="11" t="str">
+      <c r="G3" s="12" t="str">
         <f aca="false">IF(OR(E3="",E3="!!!"),"",IF(OR(J3=0,AND(J3=1,K3=1),AND(J3=1,I3="SBJ"),AND(J3=1,I3=0)),"?IN_FOCUS",IF(J3&lt;=2,"?ACTIVATED",IF(J3&lt;&gt;"","?FAMILIAR",IF(F3="NEW",IF(ISNA(VLOOKUP(E3,#REF!,1,FALSE())),"?TYPE_IDENTIFIABLE","?REFERENTIAL"),"_")))))</f>
         <v/>
       </c>
-      <c r="H3" s="12" t="str">
+      <c r="H3" s="13" t="str">
         <f aca="false">IF(J3&lt;&gt;1,"",IF(I3="SBJ","CB","?"))</f>
         <v/>
       </c>
-      <c r="I3" s="13" t="str">
+      <c r="I3" s="14" t="str">
         <f aca="false">IF(OR(E3="",E3="!!!",F3="NEW"),"",INDEX(B$2:B2,-1+SUMPRODUCT(MAX(ROW(E$2:E2)*(E3=E$2:E2)))))</f>
         <v/>
       </c>
-      <c r="J3" s="14" t="str">
+      <c r="J3" s="15" t="str">
         <f aca="true">IF(OR(E3="",E3="!!!",F3="NEW"),"",COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$2:E3)*(E3=E$2:E3)))))-COUNTBLANK(OFFSET(A$1,,,SUMPRODUCT(MAX(ROW(E$1:E2)*(E3=E$1:E2))))))</f>
         <v/>
       </c>
-      <c r="K3" s="14" t="str">
+      <c r="K3" s="15" t="str">
         <f aca="false">IF(OR(E3="",E3="!!!",F3="NEW"),"",INDEX(J$1:J2,SUMPRODUCT(MAX(ROW(E$1:E2)*(E3=E$1:E2)))))</f>
         <v/>
       </c>
+      <c r="L3" s="16"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>